<commit_message>
feat(hierarchy): remove chemical-name level filtration and integrate terminal scientific subgroup analytics
</commit_message>
<xml_diff>
--- a/outputs/debug_canonical_smiles.xlsx
+++ b/outputs/debug_canonical_smiles.xlsx
@@ -34,22 +34,22 @@
     <t>id_type</t>
   </si>
   <si>
+    <t>CC(=O)NC1=CC=C(C=C1)O</t>
+  </si>
+  <si>
     <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
   </si>
   <si>
-    <t>CC(=O)NC1=CC=C(C=C1)O</t>
+    <t>CC(=O)Nc1ccc(O)cc1</t>
   </si>
   <si>
     <t>CC(=O)Oc1ccccc1C(=O)O</t>
   </si>
   <si>
-    <t>CC(=O)Nc1ccc(O)cc1</t>
+    <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
-  </si>
-  <si>
-    <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>success</t>

</xml_diff>

<commit_message>
feat: implement scientific intelligence workspace, fix ML readiness crashes & discovery graph rendering, restore E2E verification search inputs, and update next-step workspace navigation button
</commit_message>
<xml_diff>
--- a/outputs/debug_canonical_smiles.xlsx
+++ b/outputs/debug_canonical_smiles.xlsx
@@ -34,22 +34,22 @@
     <t>id_type</t>
   </si>
   <si>
+    <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+  </si>
+  <si>
     <t>CC(=O)NC1=CC=C(C=C1)O</t>
   </si>
   <si>
-    <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+    <t>CC(=O)Oc1ccccc1C(=O)O</t>
   </si>
   <si>
     <t>CC(=O)Nc1ccc(O)cc1</t>
   </si>
   <si>
-    <t>CC(=O)Oc1ccccc1C(=O)O</t>
+    <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
-  </si>
-  <si>
-    <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>success</t>

</xml_diff>

<commit_message>
docs: push debug canonical smiles sheet deliverables
</commit_message>
<xml_diff>
--- a/outputs/debug_canonical_smiles.xlsx
+++ b/outputs/debug_canonical_smiles.xlsx
@@ -34,22 +34,22 @@
     <t>id_type</t>
   </si>
   <si>
+    <t>CC(=O)NC1=CC=C(C=C1)O</t>
+  </si>
+  <si>
     <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
   </si>
   <si>
-    <t>CC(=O)NC1=CC=C(C=C1)O</t>
+    <t>CC(=O)Nc1ccc(O)cc1</t>
   </si>
   <si>
     <t>CC(=O)Oc1ccccc1C(=O)O</t>
   </si>
   <si>
-    <t>CC(=O)Nc1ccc(O)cc1</t>
+    <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
-  </si>
-  <si>
-    <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>success</t>

</xml_diff>

<commit_message>
feat: complete SUTRIX V6 unit normalization, QSAR readiness, UI and report compiler
</commit_message>
<xml_diff>
--- a/outputs/debug_canonical_smiles.xlsx
+++ b/outputs/debug_canonical_smiles.xlsx
@@ -34,22 +34,22 @@
     <t>id_type</t>
   </si>
   <si>
+    <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+  </si>
+  <si>
     <t>CC(=O)NC1=CC=C(C=C1)O</t>
   </si>
   <si>
-    <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+    <t>CC(=O)Oc1ccccc1C(=O)O</t>
   </si>
   <si>
     <t>CC(=O)Nc1ccc(O)cc1</t>
   </si>
   <si>
-    <t>CC(=O)Oc1ccccc1C(=O)O</t>
+    <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
-  </si>
-  <si>
-    <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>success</t>

</xml_diff>

<commit_message>
feat: complete SUTRIX V6 unit normalization, QSAR readiness, UI and thesis compiler
</commit_message>
<xml_diff>
--- a/outputs/debug_canonical_smiles.xlsx
+++ b/outputs/debug_canonical_smiles.xlsx
@@ -34,22 +34,22 @@
     <t>id_type</t>
   </si>
   <si>
+    <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+  </si>
+  <si>
     <t>CC(=O)NC1=CC=C(C=C1)O</t>
   </si>
   <si>
-    <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+    <t>CC(=O)Oc1ccccc1C(=O)O</t>
   </si>
   <si>
     <t>CC(=O)Nc1ccc(O)cc1</t>
   </si>
   <si>
-    <t>CC(=O)Oc1ccccc1C(=O)O</t>
+    <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>RZVAJINKPMORJF-UHFFFAOYSA-N</t>
-  </si>
-  <si>
-    <t>BSYNRYMUTXBXSQ-UHFFFAOYSA-N</t>
   </si>
   <si>
     <t>success</t>

</xml_diff>